<commit_message>
CLRA registers: purpose-keyed templates, per-site employer forms, audited master-header field mappings
- RegisterFieldMapping keys now pin to the exact master-sheet headers (Employee_Code, Gross_Wages, Net_Salary, ...) so admin shows the real columns and renders resolve via HEADER_ALIASES (both header and canonical key work)
- Remove the redundant Remarks mapping; add Family_Pension/from_26th_days mappings and matching dual-master logic for form code remapping
- Apply to every state's templates (216 templates / 2338 columns across 32 states seeded); calc rules normalize headers to canonical keys
- Models/migrations: RegisterTemplate purpose column, CustomFormName per-site scope, employer form selection per site
</commit_message>
<xml_diff>
--- a/FINAL/Requirements/ContractorMasterSheet_Populated_4444444444.xlsx
+++ b/FINAL/Requirements/ContractorMasterSheet_Populated_4444444444.xlsx
@@ -1097,7 +1097,6 @@
           <t>Advance_Repaid_Amount</t>
         </is>
       </c>
-      <c r="EG1" t="inlineStr"/>
       <c r="EH1" t="inlineStr">
         <is>
           <t>Day1</t>
@@ -1520,7 +1519,6 @@
           <t>2023-01-10</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
           <t>Electrician</t>
@@ -1531,13 +1529,11 @@
           <t>Electrical</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr">
         <is>
           <t>Demo Metro Site</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr">
         <is>
           <t>Demo Metro Site</t>
@@ -1568,44 +1564,16 @@
           <t>Demo Contractor Pvt Ltd</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr"/>
-      <c r="V2" t="inlineStr"/>
-      <c r="W2" t="inlineStr"/>
-      <c r="X2" t="inlineStr"/>
-      <c r="Y2" t="inlineStr"/>
-      <c r="Z2" t="inlineStr"/>
-      <c r="AA2" t="inlineStr"/>
-      <c r="AB2" t="inlineStr"/>
-      <c r="AC2" t="inlineStr"/>
-      <c r="AD2" t="inlineStr"/>
       <c r="AE2" t="inlineStr">
         <is>
           <t>26</t>
         </is>
       </c>
-      <c r="AF2" t="inlineStr"/>
-      <c r="AG2" t="inlineStr"/>
-      <c r="AH2" t="inlineStr"/>
-      <c r="AI2" t="inlineStr"/>
-      <c r="AJ2" t="inlineStr"/>
-      <c r="AK2" t="inlineStr"/>
-      <c r="AL2" t="inlineStr"/>
-      <c r="AM2" t="inlineStr"/>
-      <c r="AN2" t="inlineStr"/>
-      <c r="AO2" t="inlineStr"/>
-      <c r="AP2" t="inlineStr"/>
       <c r="AQ2" t="inlineStr">
         <is>
           <t>12000</t>
         </is>
       </c>
-      <c r="AR2" t="inlineStr"/>
-      <c r="AS2" t="inlineStr"/>
-      <c r="AT2" t="inlineStr"/>
-      <c r="AU2" t="inlineStr"/>
-      <c r="AV2" t="inlineStr"/>
-      <c r="AW2" t="inlineStr"/>
       <c r="AX2" t="inlineStr">
         <is>
           <t>12000</t>
@@ -1616,18 +1584,6 @@
           <t>12000</t>
         </is>
       </c>
-      <c r="AZ2" t="inlineStr"/>
-      <c r="BA2" t="inlineStr"/>
-      <c r="BB2" t="inlineStr"/>
-      <c r="BC2" t="inlineStr"/>
-      <c r="BD2" t="inlineStr"/>
-      <c r="BE2" t="inlineStr"/>
-      <c r="BF2" t="inlineStr"/>
-      <c r="BG2" t="inlineStr"/>
-      <c r="BH2" t="inlineStr"/>
-      <c r="BI2" t="inlineStr"/>
-      <c r="BJ2" t="inlineStr"/>
-      <c r="BK2" t="inlineStr"/>
       <c r="BL2" t="inlineStr">
         <is>
           <t>12000</t>
@@ -1638,86 +1594,16 @@
           <t>1000</t>
         </is>
       </c>
-      <c r="BN2" t="inlineStr"/>
-      <c r="BO2" t="inlineStr"/>
-      <c r="BP2" t="inlineStr"/>
-      <c r="BQ2" t="inlineStr"/>
-      <c r="BR2" t="inlineStr"/>
-      <c r="BS2" t="inlineStr"/>
-      <c r="BT2" t="inlineStr"/>
-      <c r="BU2" t="inlineStr"/>
-      <c r="BV2" t="inlineStr"/>
-      <c r="BW2" t="inlineStr"/>
-      <c r="BX2" t="inlineStr"/>
-      <c r="BY2" t="inlineStr"/>
-      <c r="BZ2" t="inlineStr"/>
-      <c r="CA2" t="inlineStr"/>
-      <c r="CB2" t="inlineStr"/>
       <c r="CC2" t="inlineStr">
         <is>
           <t>1000</t>
         </is>
       </c>
-      <c r="CD2" t="inlineStr"/>
       <c r="CE2" t="inlineStr">
         <is>
           <t>11000</t>
         </is>
       </c>
-      <c r="CF2" t="inlineStr"/>
-      <c r="CG2" t="inlineStr"/>
-      <c r="CH2" t="inlineStr"/>
-      <c r="CI2" t="inlineStr"/>
-      <c r="CJ2" t="inlineStr"/>
-      <c r="CK2" t="inlineStr"/>
-      <c r="CL2" t="inlineStr"/>
-      <c r="CM2" t="inlineStr"/>
-      <c r="CN2" t="inlineStr"/>
-      <c r="CO2" t="inlineStr"/>
-      <c r="CP2" t="inlineStr"/>
-      <c r="CQ2" t="inlineStr"/>
-      <c r="CR2" t="inlineStr"/>
-      <c r="CS2" t="inlineStr"/>
-      <c r="CT2" t="inlineStr"/>
-      <c r="CU2" t="inlineStr"/>
-      <c r="CV2" t="inlineStr"/>
-      <c r="CW2" t="inlineStr"/>
-      <c r="CX2" t="inlineStr"/>
-      <c r="CY2" t="inlineStr"/>
-      <c r="CZ2" t="inlineStr"/>
-      <c r="DA2" t="inlineStr"/>
-      <c r="DB2" t="inlineStr"/>
-      <c r="DC2" t="inlineStr"/>
-      <c r="DD2" t="inlineStr"/>
-      <c r="DE2" t="inlineStr"/>
-      <c r="DF2" t="inlineStr"/>
-      <c r="DG2" t="inlineStr"/>
-      <c r="DH2" t="inlineStr"/>
-      <c r="DI2" t="inlineStr"/>
-      <c r="DJ2" t="inlineStr"/>
-      <c r="DK2" t="inlineStr"/>
-      <c r="DL2" t="inlineStr"/>
-      <c r="DM2" t="inlineStr"/>
-      <c r="DN2" t="inlineStr"/>
-      <c r="DO2" t="inlineStr"/>
-      <c r="DP2" t="inlineStr"/>
-      <c r="DQ2" t="inlineStr"/>
-      <c r="DR2" t="inlineStr"/>
-      <c r="DS2" t="inlineStr"/>
-      <c r="DT2" t="inlineStr"/>
-      <c r="DU2" t="inlineStr"/>
-      <c r="DV2" t="inlineStr"/>
-      <c r="DW2" t="inlineStr"/>
-      <c r="DX2" t="inlineStr"/>
-      <c r="DY2" t="inlineStr"/>
-      <c r="DZ2" t="inlineStr"/>
-      <c r="EA2" t="inlineStr"/>
-      <c r="EB2" t="inlineStr"/>
-      <c r="EC2" t="inlineStr"/>
-      <c r="ED2" t="inlineStr"/>
-      <c r="EE2" t="inlineStr"/>
-      <c r="EF2" t="inlineStr"/>
-      <c r="EG2" t="inlineStr"/>
       <c r="EH2" t="inlineStr">
         <is>
           <t>P</t>
@@ -1873,60 +1759,16 @@
           <t>P</t>
         </is>
       </c>
-      <c r="FM2" t="inlineStr"/>
-      <c r="FN2" t="inlineStr"/>
-      <c r="FO2" t="inlineStr"/>
-      <c r="FP2" t="inlineStr"/>
-      <c r="FQ2" t="inlineStr"/>
-      <c r="FR2" t="inlineStr"/>
-      <c r="FS2" t="inlineStr"/>
-      <c r="FT2" t="inlineStr"/>
-      <c r="FU2" t="inlineStr"/>
-      <c r="FV2" t="inlineStr"/>
-      <c r="FW2" t="inlineStr"/>
-      <c r="FX2" t="inlineStr"/>
-      <c r="FY2" t="inlineStr"/>
-      <c r="FZ2" t="inlineStr"/>
-      <c r="GA2" t="inlineStr"/>
-      <c r="GB2" t="inlineStr"/>
-      <c r="GC2" t="inlineStr"/>
-      <c r="GD2" t="inlineStr"/>
-      <c r="GE2" t="inlineStr"/>
-      <c r="GF2" t="inlineStr"/>
-      <c r="GG2" t="inlineStr"/>
-      <c r="GH2" t="inlineStr"/>
-      <c r="GI2" t="inlineStr"/>
-      <c r="GJ2" t="inlineStr"/>
-      <c r="GK2" t="inlineStr"/>
-      <c r="GL2" t="inlineStr"/>
-      <c r="GM2" t="inlineStr"/>
-      <c r="GN2" t="inlineStr"/>
-      <c r="GO2" t="inlineStr"/>
-      <c r="GP2" t="inlineStr"/>
-      <c r="GQ2" t="inlineStr"/>
-      <c r="GR2" t="inlineStr"/>
-      <c r="GS2" t="inlineStr"/>
-      <c r="GT2" t="inlineStr"/>
-      <c r="GU2" t="inlineStr"/>
-      <c r="GV2" t="inlineStr"/>
-      <c r="GW2" t="inlineStr"/>
-      <c r="GX2" t="inlineStr"/>
-      <c r="GY2" t="inlineStr"/>
-      <c r="GZ2" t="inlineStr"/>
-      <c r="HA2" t="inlineStr"/>
       <c r="HB2" t="inlineStr">
         <is>
           <t>TS001</t>
         </is>
       </c>
-      <c r="HC2" t="inlineStr"/>
       <c r="HD2" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="HE2" t="inlineStr"/>
-      <c r="HF2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1964,7 +1806,6 @@
           <t>2023-03-15</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
           <t>Helper</t>
@@ -1975,16 +1816,14 @@
           <t>Civil</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Demo Highway Site</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr"/>
+          <t>Demo Metro Site</t>
+        </is>
+      </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Demo Highway Site</t>
+          <t>Demo Metro Site</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -2012,44 +1851,16 @@
           <t>Demo Contractor Pvt Ltd</t>
         </is>
       </c>
-      <c r="T3" t="inlineStr"/>
-      <c r="U3" t="inlineStr"/>
-      <c r="V3" t="inlineStr"/>
-      <c r="W3" t="inlineStr"/>
-      <c r="X3" t="inlineStr"/>
-      <c r="Y3" t="inlineStr"/>
-      <c r="Z3" t="inlineStr"/>
-      <c r="AA3" t="inlineStr"/>
-      <c r="AB3" t="inlineStr"/>
-      <c r="AC3" t="inlineStr"/>
-      <c r="AD3" t="inlineStr"/>
       <c r="AE3" t="inlineStr">
         <is>
           <t>25</t>
         </is>
       </c>
-      <c r="AF3" t="inlineStr"/>
-      <c r="AG3" t="inlineStr"/>
-      <c r="AH3" t="inlineStr"/>
-      <c r="AI3" t="inlineStr"/>
-      <c r="AJ3" t="inlineStr"/>
-      <c r="AK3" t="inlineStr"/>
-      <c r="AL3" t="inlineStr"/>
-      <c r="AM3" t="inlineStr"/>
-      <c r="AN3" t="inlineStr"/>
-      <c r="AO3" t="inlineStr"/>
-      <c r="AP3" t="inlineStr"/>
       <c r="AQ3" t="inlineStr">
         <is>
           <t>10000</t>
         </is>
       </c>
-      <c r="AR3" t="inlineStr"/>
-      <c r="AS3" t="inlineStr"/>
-      <c r="AT3" t="inlineStr"/>
-      <c r="AU3" t="inlineStr"/>
-      <c r="AV3" t="inlineStr"/>
-      <c r="AW3" t="inlineStr"/>
       <c r="AX3" t="inlineStr">
         <is>
           <t>10000</t>
@@ -2060,18 +1871,6 @@
           <t>10000</t>
         </is>
       </c>
-      <c r="AZ3" t="inlineStr"/>
-      <c r="BA3" t="inlineStr"/>
-      <c r="BB3" t="inlineStr"/>
-      <c r="BC3" t="inlineStr"/>
-      <c r="BD3" t="inlineStr"/>
-      <c r="BE3" t="inlineStr"/>
-      <c r="BF3" t="inlineStr"/>
-      <c r="BG3" t="inlineStr"/>
-      <c r="BH3" t="inlineStr"/>
-      <c r="BI3" t="inlineStr"/>
-      <c r="BJ3" t="inlineStr"/>
-      <c r="BK3" t="inlineStr"/>
       <c r="BL3" t="inlineStr">
         <is>
           <t>10000</t>
@@ -2082,86 +1881,16 @@
           <t>800</t>
         </is>
       </c>
-      <c r="BN3" t="inlineStr"/>
-      <c r="BO3" t="inlineStr"/>
-      <c r="BP3" t="inlineStr"/>
-      <c r="BQ3" t="inlineStr"/>
-      <c r="BR3" t="inlineStr"/>
-      <c r="BS3" t="inlineStr"/>
-      <c r="BT3" t="inlineStr"/>
-      <c r="BU3" t="inlineStr"/>
-      <c r="BV3" t="inlineStr"/>
-      <c r="BW3" t="inlineStr"/>
-      <c r="BX3" t="inlineStr"/>
-      <c r="BY3" t="inlineStr"/>
-      <c r="BZ3" t="inlineStr"/>
-      <c r="CA3" t="inlineStr"/>
-      <c r="CB3" t="inlineStr"/>
       <c r="CC3" t="inlineStr">
         <is>
           <t>800</t>
         </is>
       </c>
-      <c r="CD3" t="inlineStr"/>
       <c r="CE3" t="inlineStr">
         <is>
           <t>9200</t>
         </is>
       </c>
-      <c r="CF3" t="inlineStr"/>
-      <c r="CG3" t="inlineStr"/>
-      <c r="CH3" t="inlineStr"/>
-      <c r="CI3" t="inlineStr"/>
-      <c r="CJ3" t="inlineStr"/>
-      <c r="CK3" t="inlineStr"/>
-      <c r="CL3" t="inlineStr"/>
-      <c r="CM3" t="inlineStr"/>
-      <c r="CN3" t="inlineStr"/>
-      <c r="CO3" t="inlineStr"/>
-      <c r="CP3" t="inlineStr"/>
-      <c r="CQ3" t="inlineStr"/>
-      <c r="CR3" t="inlineStr"/>
-      <c r="CS3" t="inlineStr"/>
-      <c r="CT3" t="inlineStr"/>
-      <c r="CU3" t="inlineStr"/>
-      <c r="CV3" t="inlineStr"/>
-      <c r="CW3" t="inlineStr"/>
-      <c r="CX3" t="inlineStr"/>
-      <c r="CY3" t="inlineStr"/>
-      <c r="CZ3" t="inlineStr"/>
-      <c r="DA3" t="inlineStr"/>
-      <c r="DB3" t="inlineStr"/>
-      <c r="DC3" t="inlineStr"/>
-      <c r="DD3" t="inlineStr"/>
-      <c r="DE3" t="inlineStr"/>
-      <c r="DF3" t="inlineStr"/>
-      <c r="DG3" t="inlineStr"/>
-      <c r="DH3" t="inlineStr"/>
-      <c r="DI3" t="inlineStr"/>
-      <c r="DJ3" t="inlineStr"/>
-      <c r="DK3" t="inlineStr"/>
-      <c r="DL3" t="inlineStr"/>
-      <c r="DM3" t="inlineStr"/>
-      <c r="DN3" t="inlineStr"/>
-      <c r="DO3" t="inlineStr"/>
-      <c r="DP3" t="inlineStr"/>
-      <c r="DQ3" t="inlineStr"/>
-      <c r="DR3" t="inlineStr"/>
-      <c r="DS3" t="inlineStr"/>
-      <c r="DT3" t="inlineStr"/>
-      <c r="DU3" t="inlineStr"/>
-      <c r="DV3" t="inlineStr"/>
-      <c r="DW3" t="inlineStr"/>
-      <c r="DX3" t="inlineStr"/>
-      <c r="DY3" t="inlineStr"/>
-      <c r="DZ3" t="inlineStr"/>
-      <c r="EA3" t="inlineStr"/>
-      <c r="EB3" t="inlineStr"/>
-      <c r="EC3" t="inlineStr"/>
-      <c r="ED3" t="inlineStr"/>
-      <c r="EE3" t="inlineStr"/>
-      <c r="EF3" t="inlineStr"/>
-      <c r="EG3" t="inlineStr"/>
       <c r="EH3" t="inlineStr">
         <is>
           <t>P</t>
@@ -2317,60 +2046,16 @@
           <t>P</t>
         </is>
       </c>
-      <c r="FM3" t="inlineStr"/>
-      <c r="FN3" t="inlineStr"/>
-      <c r="FO3" t="inlineStr"/>
-      <c r="FP3" t="inlineStr"/>
-      <c r="FQ3" t="inlineStr"/>
-      <c r="FR3" t="inlineStr"/>
-      <c r="FS3" t="inlineStr"/>
-      <c r="FT3" t="inlineStr"/>
-      <c r="FU3" t="inlineStr"/>
-      <c r="FV3" t="inlineStr"/>
-      <c r="FW3" t="inlineStr"/>
-      <c r="FX3" t="inlineStr"/>
-      <c r="FY3" t="inlineStr"/>
-      <c r="FZ3" t="inlineStr"/>
-      <c r="GA3" t="inlineStr"/>
-      <c r="GB3" t="inlineStr"/>
-      <c r="GC3" t="inlineStr"/>
-      <c r="GD3" t="inlineStr"/>
-      <c r="GE3" t="inlineStr"/>
-      <c r="GF3" t="inlineStr"/>
-      <c r="GG3" t="inlineStr"/>
-      <c r="GH3" t="inlineStr"/>
-      <c r="GI3" t="inlineStr"/>
-      <c r="GJ3" t="inlineStr"/>
-      <c r="GK3" t="inlineStr"/>
-      <c r="GL3" t="inlineStr"/>
-      <c r="GM3" t="inlineStr"/>
-      <c r="GN3" t="inlineStr"/>
-      <c r="GO3" t="inlineStr"/>
-      <c r="GP3" t="inlineStr"/>
-      <c r="GQ3" t="inlineStr"/>
-      <c r="GR3" t="inlineStr"/>
-      <c r="GS3" t="inlineStr"/>
-      <c r="GT3" t="inlineStr"/>
-      <c r="GU3" t="inlineStr"/>
-      <c r="GV3" t="inlineStr"/>
-      <c r="GW3" t="inlineStr"/>
-      <c r="GX3" t="inlineStr"/>
-      <c r="GY3" t="inlineStr"/>
-      <c r="GZ3" t="inlineStr"/>
-      <c r="HA3" t="inlineStr"/>
       <c r="HB3" t="inlineStr">
         <is>
-          <t>TS002</t>
-        </is>
-      </c>
-      <c r="HC3" t="inlineStr"/>
+          <t>TS001</t>
+        </is>
+      </c>
       <c r="HD3" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="HE3" t="inlineStr"/>
-      <c r="HF3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2408,7 +2093,6 @@
           <t>2022-11-01</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
         <is>
           <t>Mason</t>
@@ -2419,21 +2103,19 @@
           <t>Civil</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr">
         <is>
-          <t>AP Construction Site</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr"/>
+          <t>Demo Metro Site</t>
+        </is>
+      </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>AP Construction Site</t>
+          <t>Demo Metro Site</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Andhra Pradesh</t>
+          <t>Maharashtra</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
@@ -2456,44 +2138,16 @@
           <t>Demo Contractor Pvt Ltd</t>
         </is>
       </c>
-      <c r="T4" t="inlineStr"/>
-      <c r="U4" t="inlineStr"/>
-      <c r="V4" t="inlineStr"/>
-      <c r="W4" t="inlineStr"/>
-      <c r="X4" t="inlineStr"/>
-      <c r="Y4" t="inlineStr"/>
-      <c r="Z4" t="inlineStr"/>
-      <c r="AA4" t="inlineStr"/>
-      <c r="AB4" t="inlineStr"/>
-      <c r="AC4" t="inlineStr"/>
-      <c r="AD4" t="inlineStr"/>
       <c r="AE4" t="inlineStr">
         <is>
           <t>26</t>
         </is>
       </c>
-      <c r="AF4" t="inlineStr"/>
-      <c r="AG4" t="inlineStr"/>
-      <c r="AH4" t="inlineStr"/>
-      <c r="AI4" t="inlineStr"/>
-      <c r="AJ4" t="inlineStr"/>
-      <c r="AK4" t="inlineStr"/>
-      <c r="AL4" t="inlineStr"/>
-      <c r="AM4" t="inlineStr"/>
-      <c r="AN4" t="inlineStr"/>
-      <c r="AO4" t="inlineStr"/>
-      <c r="AP4" t="inlineStr"/>
       <c r="AQ4" t="inlineStr">
         <is>
           <t>15000</t>
         </is>
       </c>
-      <c r="AR4" t="inlineStr"/>
-      <c r="AS4" t="inlineStr"/>
-      <c r="AT4" t="inlineStr"/>
-      <c r="AU4" t="inlineStr"/>
-      <c r="AV4" t="inlineStr"/>
-      <c r="AW4" t="inlineStr"/>
       <c r="AX4" t="inlineStr">
         <is>
           <t>15000</t>
@@ -2504,18 +2158,6 @@
           <t>15000</t>
         </is>
       </c>
-      <c r="AZ4" t="inlineStr"/>
-      <c r="BA4" t="inlineStr"/>
-      <c r="BB4" t="inlineStr"/>
-      <c r="BC4" t="inlineStr"/>
-      <c r="BD4" t="inlineStr"/>
-      <c r="BE4" t="inlineStr"/>
-      <c r="BF4" t="inlineStr"/>
-      <c r="BG4" t="inlineStr"/>
-      <c r="BH4" t="inlineStr"/>
-      <c r="BI4" t="inlineStr"/>
-      <c r="BJ4" t="inlineStr"/>
-      <c r="BK4" t="inlineStr"/>
       <c r="BL4" t="inlineStr">
         <is>
           <t>15000</t>
@@ -2526,86 +2168,16 @@
           <t>1200</t>
         </is>
       </c>
-      <c r="BN4" t="inlineStr"/>
-      <c r="BO4" t="inlineStr"/>
-      <c r="BP4" t="inlineStr"/>
-      <c r="BQ4" t="inlineStr"/>
-      <c r="BR4" t="inlineStr"/>
-      <c r="BS4" t="inlineStr"/>
-      <c r="BT4" t="inlineStr"/>
-      <c r="BU4" t="inlineStr"/>
-      <c r="BV4" t="inlineStr"/>
-      <c r="BW4" t="inlineStr"/>
-      <c r="BX4" t="inlineStr"/>
-      <c r="BY4" t="inlineStr"/>
-      <c r="BZ4" t="inlineStr"/>
-      <c r="CA4" t="inlineStr"/>
-      <c r="CB4" t="inlineStr"/>
       <c r="CC4" t="inlineStr">
         <is>
           <t>1200</t>
         </is>
       </c>
-      <c r="CD4" t="inlineStr"/>
       <c r="CE4" t="inlineStr">
         <is>
           <t>13800</t>
         </is>
       </c>
-      <c r="CF4" t="inlineStr"/>
-      <c r="CG4" t="inlineStr"/>
-      <c r="CH4" t="inlineStr"/>
-      <c r="CI4" t="inlineStr"/>
-      <c r="CJ4" t="inlineStr"/>
-      <c r="CK4" t="inlineStr"/>
-      <c r="CL4" t="inlineStr"/>
-      <c r="CM4" t="inlineStr"/>
-      <c r="CN4" t="inlineStr"/>
-      <c r="CO4" t="inlineStr"/>
-      <c r="CP4" t="inlineStr"/>
-      <c r="CQ4" t="inlineStr"/>
-      <c r="CR4" t="inlineStr"/>
-      <c r="CS4" t="inlineStr"/>
-      <c r="CT4" t="inlineStr"/>
-      <c r="CU4" t="inlineStr"/>
-      <c r="CV4" t="inlineStr"/>
-      <c r="CW4" t="inlineStr"/>
-      <c r="CX4" t="inlineStr"/>
-      <c r="CY4" t="inlineStr"/>
-      <c r="CZ4" t="inlineStr"/>
-      <c r="DA4" t="inlineStr"/>
-      <c r="DB4" t="inlineStr"/>
-      <c r="DC4" t="inlineStr"/>
-      <c r="DD4" t="inlineStr"/>
-      <c r="DE4" t="inlineStr"/>
-      <c r="DF4" t="inlineStr"/>
-      <c r="DG4" t="inlineStr"/>
-      <c r="DH4" t="inlineStr"/>
-      <c r="DI4" t="inlineStr"/>
-      <c r="DJ4" t="inlineStr"/>
-      <c r="DK4" t="inlineStr"/>
-      <c r="DL4" t="inlineStr"/>
-      <c r="DM4" t="inlineStr"/>
-      <c r="DN4" t="inlineStr"/>
-      <c r="DO4" t="inlineStr"/>
-      <c r="DP4" t="inlineStr"/>
-      <c r="DQ4" t="inlineStr"/>
-      <c r="DR4" t="inlineStr"/>
-      <c r="DS4" t="inlineStr"/>
-      <c r="DT4" t="inlineStr"/>
-      <c r="DU4" t="inlineStr"/>
-      <c r="DV4" t="inlineStr"/>
-      <c r="DW4" t="inlineStr"/>
-      <c r="DX4" t="inlineStr"/>
-      <c r="DY4" t="inlineStr"/>
-      <c r="DZ4" t="inlineStr"/>
-      <c r="EA4" t="inlineStr"/>
-      <c r="EB4" t="inlineStr"/>
-      <c r="EC4" t="inlineStr"/>
-      <c r="ED4" t="inlineStr"/>
-      <c r="EE4" t="inlineStr"/>
-      <c r="EF4" t="inlineStr"/>
-      <c r="EG4" t="inlineStr"/>
       <c r="EH4" t="inlineStr">
         <is>
           <t>P</t>
@@ -2761,60 +2333,16 @@
           <t>P</t>
         </is>
       </c>
-      <c r="FM4" t="inlineStr"/>
-      <c r="FN4" t="inlineStr"/>
-      <c r="FO4" t="inlineStr"/>
-      <c r="FP4" t="inlineStr"/>
-      <c r="FQ4" t="inlineStr"/>
-      <c r="FR4" t="inlineStr"/>
-      <c r="FS4" t="inlineStr"/>
-      <c r="FT4" t="inlineStr"/>
-      <c r="FU4" t="inlineStr"/>
-      <c r="FV4" t="inlineStr"/>
-      <c r="FW4" t="inlineStr"/>
-      <c r="FX4" t="inlineStr"/>
-      <c r="FY4" t="inlineStr"/>
-      <c r="FZ4" t="inlineStr"/>
-      <c r="GA4" t="inlineStr"/>
-      <c r="GB4" t="inlineStr"/>
-      <c r="GC4" t="inlineStr"/>
-      <c r="GD4" t="inlineStr"/>
-      <c r="GE4" t="inlineStr"/>
-      <c r="GF4" t="inlineStr"/>
-      <c r="GG4" t="inlineStr"/>
-      <c r="GH4" t="inlineStr"/>
-      <c r="GI4" t="inlineStr"/>
-      <c r="GJ4" t="inlineStr"/>
-      <c r="GK4" t="inlineStr"/>
-      <c r="GL4" t="inlineStr"/>
-      <c r="GM4" t="inlineStr"/>
-      <c r="GN4" t="inlineStr"/>
-      <c r="GO4" t="inlineStr"/>
-      <c r="GP4" t="inlineStr"/>
-      <c r="GQ4" t="inlineStr"/>
-      <c r="GR4" t="inlineStr"/>
-      <c r="GS4" t="inlineStr"/>
-      <c r="GT4" t="inlineStr"/>
-      <c r="GU4" t="inlineStr"/>
-      <c r="GV4" t="inlineStr"/>
-      <c r="GW4" t="inlineStr"/>
-      <c r="GX4" t="inlineStr"/>
-      <c r="GY4" t="inlineStr"/>
-      <c r="GZ4" t="inlineStr"/>
-      <c r="HA4" t="inlineStr"/>
       <c r="HB4" t="inlineStr">
         <is>
-          <t>AP001</t>
-        </is>
-      </c>
-      <c r="HC4" t="inlineStr"/>
+          <t>TS001</t>
+        </is>
+      </c>
       <c r="HD4" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="HE4" t="inlineStr"/>
-      <c r="HF4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2852,7 +2380,6 @@
           <t>2024-01-05</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
           <t>Welder</t>
@@ -2863,21 +2390,19 @@
           <t>Mechanical</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
-          <t>AP Construction Site</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr"/>
+          <t>Demo Metro Site</t>
+        </is>
+      </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>AP Construction Site</t>
+          <t>Demo Metro Site</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Andhra Pradesh</t>
+          <t>Maharashtra</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
@@ -2900,44 +2425,16 @@
           <t>Demo Contractor Pvt Ltd</t>
         </is>
       </c>
-      <c r="T5" t="inlineStr"/>
-      <c r="U5" t="inlineStr"/>
-      <c r="V5" t="inlineStr"/>
-      <c r="W5" t="inlineStr"/>
-      <c r="X5" t="inlineStr"/>
-      <c r="Y5" t="inlineStr"/>
-      <c r="Z5" t="inlineStr"/>
-      <c r="AA5" t="inlineStr"/>
-      <c r="AB5" t="inlineStr"/>
-      <c r="AC5" t="inlineStr"/>
-      <c r="AD5" t="inlineStr"/>
       <c r="AE5" t="inlineStr">
         <is>
           <t>24</t>
         </is>
       </c>
-      <c r="AF5" t="inlineStr"/>
-      <c r="AG5" t="inlineStr"/>
-      <c r="AH5" t="inlineStr"/>
-      <c r="AI5" t="inlineStr"/>
-      <c r="AJ5" t="inlineStr"/>
-      <c r="AK5" t="inlineStr"/>
-      <c r="AL5" t="inlineStr"/>
-      <c r="AM5" t="inlineStr"/>
-      <c r="AN5" t="inlineStr"/>
-      <c r="AO5" t="inlineStr"/>
-      <c r="AP5" t="inlineStr"/>
       <c r="AQ5" t="inlineStr">
         <is>
           <t>14000</t>
         </is>
       </c>
-      <c r="AR5" t="inlineStr"/>
-      <c r="AS5" t="inlineStr"/>
-      <c r="AT5" t="inlineStr"/>
-      <c r="AU5" t="inlineStr"/>
-      <c r="AV5" t="inlineStr"/>
-      <c r="AW5" t="inlineStr"/>
       <c r="AX5" t="inlineStr">
         <is>
           <t>14000</t>
@@ -2948,18 +2445,6 @@
           <t>14000</t>
         </is>
       </c>
-      <c r="AZ5" t="inlineStr"/>
-      <c r="BA5" t="inlineStr"/>
-      <c r="BB5" t="inlineStr"/>
-      <c r="BC5" t="inlineStr"/>
-      <c r="BD5" t="inlineStr"/>
-      <c r="BE5" t="inlineStr"/>
-      <c r="BF5" t="inlineStr"/>
-      <c r="BG5" t="inlineStr"/>
-      <c r="BH5" t="inlineStr"/>
-      <c r="BI5" t="inlineStr"/>
-      <c r="BJ5" t="inlineStr"/>
-      <c r="BK5" t="inlineStr"/>
       <c r="BL5" t="inlineStr">
         <is>
           <t>14000</t>
@@ -2970,86 +2455,16 @@
           <t>1100</t>
         </is>
       </c>
-      <c r="BN5" t="inlineStr"/>
-      <c r="BO5" t="inlineStr"/>
-      <c r="BP5" t="inlineStr"/>
-      <c r="BQ5" t="inlineStr"/>
-      <c r="BR5" t="inlineStr"/>
-      <c r="BS5" t="inlineStr"/>
-      <c r="BT5" t="inlineStr"/>
-      <c r="BU5" t="inlineStr"/>
-      <c r="BV5" t="inlineStr"/>
-      <c r="BW5" t="inlineStr"/>
-      <c r="BX5" t="inlineStr"/>
-      <c r="BY5" t="inlineStr"/>
-      <c r="BZ5" t="inlineStr"/>
-      <c r="CA5" t="inlineStr"/>
-      <c r="CB5" t="inlineStr"/>
       <c r="CC5" t="inlineStr">
         <is>
           <t>1100</t>
         </is>
       </c>
-      <c r="CD5" t="inlineStr"/>
       <c r="CE5" t="inlineStr">
         <is>
           <t>12900</t>
         </is>
       </c>
-      <c r="CF5" t="inlineStr"/>
-      <c r="CG5" t="inlineStr"/>
-      <c r="CH5" t="inlineStr"/>
-      <c r="CI5" t="inlineStr"/>
-      <c r="CJ5" t="inlineStr"/>
-      <c r="CK5" t="inlineStr"/>
-      <c r="CL5" t="inlineStr"/>
-      <c r="CM5" t="inlineStr"/>
-      <c r="CN5" t="inlineStr"/>
-      <c r="CO5" t="inlineStr"/>
-      <c r="CP5" t="inlineStr"/>
-      <c r="CQ5" t="inlineStr"/>
-      <c r="CR5" t="inlineStr"/>
-      <c r="CS5" t="inlineStr"/>
-      <c r="CT5" t="inlineStr"/>
-      <c r="CU5" t="inlineStr"/>
-      <c r="CV5" t="inlineStr"/>
-      <c r="CW5" t="inlineStr"/>
-      <c r="CX5" t="inlineStr"/>
-      <c r="CY5" t="inlineStr"/>
-      <c r="CZ5" t="inlineStr"/>
-      <c r="DA5" t="inlineStr"/>
-      <c r="DB5" t="inlineStr"/>
-      <c r="DC5" t="inlineStr"/>
-      <c r="DD5" t="inlineStr"/>
-      <c r="DE5" t="inlineStr"/>
-      <c r="DF5" t="inlineStr"/>
-      <c r="DG5" t="inlineStr"/>
-      <c r="DH5" t="inlineStr"/>
-      <c r="DI5" t="inlineStr"/>
-      <c r="DJ5" t="inlineStr"/>
-      <c r="DK5" t="inlineStr"/>
-      <c r="DL5" t="inlineStr"/>
-      <c r="DM5" t="inlineStr"/>
-      <c r="DN5" t="inlineStr"/>
-      <c r="DO5" t="inlineStr"/>
-      <c r="DP5" t="inlineStr"/>
-      <c r="DQ5" t="inlineStr"/>
-      <c r="DR5" t="inlineStr"/>
-      <c r="DS5" t="inlineStr"/>
-      <c r="DT5" t="inlineStr"/>
-      <c r="DU5" t="inlineStr"/>
-      <c r="DV5" t="inlineStr"/>
-      <c r="DW5" t="inlineStr"/>
-      <c r="DX5" t="inlineStr"/>
-      <c r="DY5" t="inlineStr"/>
-      <c r="DZ5" t="inlineStr"/>
-      <c r="EA5" t="inlineStr"/>
-      <c r="EB5" t="inlineStr"/>
-      <c r="EC5" t="inlineStr"/>
-      <c r="ED5" t="inlineStr"/>
-      <c r="EE5" t="inlineStr"/>
-      <c r="EF5" t="inlineStr"/>
-      <c r="EG5" t="inlineStr"/>
       <c r="EH5" t="inlineStr">
         <is>
           <t>P</t>
@@ -3205,60 +2620,16 @@
           <t>P</t>
         </is>
       </c>
-      <c r="FM5" t="inlineStr"/>
-      <c r="FN5" t="inlineStr"/>
-      <c r="FO5" t="inlineStr"/>
-      <c r="FP5" t="inlineStr"/>
-      <c r="FQ5" t="inlineStr"/>
-      <c r="FR5" t="inlineStr"/>
-      <c r="FS5" t="inlineStr"/>
-      <c r="FT5" t="inlineStr"/>
-      <c r="FU5" t="inlineStr"/>
-      <c r="FV5" t="inlineStr"/>
-      <c r="FW5" t="inlineStr"/>
-      <c r="FX5" t="inlineStr"/>
-      <c r="FY5" t="inlineStr"/>
-      <c r="FZ5" t="inlineStr"/>
-      <c r="GA5" t="inlineStr"/>
-      <c r="GB5" t="inlineStr"/>
-      <c r="GC5" t="inlineStr"/>
-      <c r="GD5" t="inlineStr"/>
-      <c r="GE5" t="inlineStr"/>
-      <c r="GF5" t="inlineStr"/>
-      <c r="GG5" t="inlineStr"/>
-      <c r="GH5" t="inlineStr"/>
-      <c r="GI5" t="inlineStr"/>
-      <c r="GJ5" t="inlineStr"/>
-      <c r="GK5" t="inlineStr"/>
-      <c r="GL5" t="inlineStr"/>
-      <c r="GM5" t="inlineStr"/>
-      <c r="GN5" t="inlineStr"/>
-      <c r="GO5" t="inlineStr"/>
-      <c r="GP5" t="inlineStr"/>
-      <c r="GQ5" t="inlineStr"/>
-      <c r="GR5" t="inlineStr"/>
-      <c r="GS5" t="inlineStr"/>
-      <c r="GT5" t="inlineStr"/>
-      <c r="GU5" t="inlineStr"/>
-      <c r="GV5" t="inlineStr"/>
-      <c r="GW5" t="inlineStr"/>
-      <c r="GX5" t="inlineStr"/>
-      <c r="GY5" t="inlineStr"/>
-      <c r="GZ5" t="inlineStr"/>
-      <c r="HA5" t="inlineStr"/>
       <c r="HB5" t="inlineStr">
         <is>
-          <t>AP001</t>
-        </is>
-      </c>
-      <c r="HC5" t="inlineStr"/>
+          <t>TS001</t>
+        </is>
+      </c>
       <c r="HD5" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="HE5" t="inlineStr"/>
-      <c r="HF5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>